<commit_message>
Remove `depends_on` from ssbt.yml and infer dependencies from SQL `{{ ref('name') }}` calls instead. Adjust related logic in README and engine.py accordingly.
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccarpenter\PycharmProjects\ssbt\ssbt\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccarpenter\PycharmProjects\ssbt\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C18D7A4-F1EB-4177-ACC0-A43D9DE2473D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5347AE83-B82E-42DD-A3C5-905E9D928C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -519,6 +519,9 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
       <c r="B7" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Handle Excel formula errors gracefully by falling back to openpyxl when `read_xlsx` fails. Improve type coercion logic and refactor imports.
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccarpenter\PycharmProjects\ssbt\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5347AE83-B82E-42DD-A3C5-905E9D928C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3763C72-C119-4122-928E-BAD665C36D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_orders" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -548,8 +561,9 @@
       <c r="D8" t="s">
         <v>7</v>
       </c>
-      <c r="E8">
-        <v>45</v>
+      <c r="E8" t="e">
+        <f>1/0</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -583,7 +597,8 @@
         <v>7</v>
       </c>
       <c r="E10">
-        <v>210</v>
+        <f>SUM(E3:E4)</f>
+        <v>275.5</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add `docs` command to generate project documentation, including DAG, models, and sources. Update README with usage instructions.
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccarpenter\PycharmProjects\ssbt\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3763C72-C119-4122-928E-BAD665C36D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B487A96C-3620-45C5-8F71-247D7A07C3BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -561,9 +561,8 @@
       <c r="D8" t="s">
         <v>7</v>
       </c>
-      <c r="E8" t="e">
-        <f>1/0</f>
-        <v>#DIV/0!</v>
+      <c r="E8">
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>